<commit_message>
Reverted, fixed elo swap bug
</commit_message>
<xml_diff>
--- a/Predictions/2026-04-18.xlsx
+++ b/Predictions/2026-04-18.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gdsak\OneDrive\Desktop\Glicko-2, Etc\Predictions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6ECE5AB-74F1-4096-9AAA-8D632D979052}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07D2CA53-D5D4-44B6-A2EC-5B71409348F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="42">
   <si>
     <t>Red Corner</t>
   </si>
@@ -137,6 +137,39 @@
   </si>
   <si>
     <t>Old Model</t>
+  </si>
+  <si>
+    <t>Submission</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">John Castaneda </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>(Draw)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Jamey-Lyn Horth </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>(Robbery)</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -146,7 +179,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -168,8 +201,15 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -182,6 +222,12 @@
         <bgColor rgb="FFD3D3D3"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="20">
     <border>
@@ -450,7 +496,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -483,64 +529,88 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="10" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="17" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -851,7 +921,7 @@
     <col min="1" max="1" width="19.7109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="19" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="23" customWidth="1"/>
-    <col min="4" max="4" width="19.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="25.5703125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="6.7109375" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="11.140625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="10.140625" bestFit="1" customWidth="1"/>
@@ -865,23 +935,23 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="D1" s="24" t="s">
+      <c r="D1" s="27" t="s">
         <v>34</v>
       </c>
-      <c r="E1" s="13"/>
-      <c r="F1" s="13"/>
-      <c r="G1" s="13"/>
-      <c r="H1" s="13"/>
-      <c r="I1" s="13"/>
-      <c r="J1" s="25"/>
-      <c r="K1" s="13" t="s">
+      <c r="E1" s="28"/>
+      <c r="F1" s="28"/>
+      <c r="G1" s="28"/>
+      <c r="H1" s="28"/>
+      <c r="I1" s="28"/>
+      <c r="J1" s="29"/>
+      <c r="K1" s="28" t="s">
         <v>38</v>
       </c>
-      <c r="L1" s="14"/>
-      <c r="M1" s="12" t="s">
+      <c r="L1" s="31"/>
+      <c r="M1" s="30" t="s">
         <v>33</v>
       </c>
-      <c r="N1" s="14"/>
+      <c r="N1" s="31"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
@@ -893,7 +963,7 @@
       <c r="C2" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="26" t="s">
+      <c r="D2" s="21" t="s">
         <v>31</v>
       </c>
       <c r="E2" s="1" t="s">
@@ -911,10 +981,10 @@
       <c r="I2" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="J2" s="27" t="s">
+      <c r="J2" s="22" t="s">
         <v>37</v>
       </c>
-      <c r="K2" s="21" t="s">
+      <c r="K2" s="18" t="s">
         <v>31</v>
       </c>
       <c r="L2" s="1" t="s">
@@ -937,37 +1007,37 @@
       <c r="C3" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="D3" s="28" t="s">
+      <c r="D3" s="36" t="s">
         <v>6</v>
       </c>
-      <c r="E3" s="3">
-        <v>0.72262345805072037</v>
-      </c>
-      <c r="F3" s="2" t="s">
+      <c r="E3" s="37">
+        <v>0.73</v>
+      </c>
+      <c r="F3" s="38" t="s">
         <v>15</v>
       </c>
-      <c r="G3" s="3">
-        <v>0.46881479893066991</v>
-      </c>
-      <c r="H3" s="3">
-        <v>0.3002394439659018</v>
-      </c>
-      <c r="I3" s="3">
-        <v>0.46881479893066991</v>
-      </c>
-      <c r="J3" s="29">
-        <v>0.2309457571034283</v>
-      </c>
-      <c r="K3" s="22" t="s">
+      <c r="G3" s="37">
+        <v>0.441</v>
+      </c>
+      <c r="H3" s="37">
+        <v>0.31</v>
+      </c>
+      <c r="I3" s="37">
+        <v>0.441</v>
+      </c>
+      <c r="J3" s="39">
+        <v>0.249</v>
+      </c>
+      <c r="K3" s="32" t="s">
         <v>6</v>
       </c>
-      <c r="L3" s="10">
+      <c r="L3" s="33">
         <v>0.58507962712671024</v>
       </c>
-      <c r="M3" s="7" t="s">
+      <c r="M3" s="34" t="s">
         <v>6</v>
       </c>
-      <c r="N3" s="8">
+      <c r="N3" s="35">
         <v>0.53724954619042453</v>
       </c>
     </row>
@@ -981,28 +1051,28 @@
       <c r="C4" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="D4" s="28" t="s">
+      <c r="D4" s="36" t="s">
         <v>10</v>
       </c>
-      <c r="E4" s="3">
-        <v>0.57901563301901415</v>
-      </c>
-      <c r="F4" s="2" t="s">
+      <c r="E4" s="37">
+        <v>0.59099999999999997</v>
+      </c>
+      <c r="F4" s="38" t="s">
         <v>8</v>
       </c>
-      <c r="G4" s="3">
-        <v>0.44842107401794429</v>
-      </c>
-      <c r="H4" s="3">
-        <v>0.44842107401794429</v>
-      </c>
-      <c r="I4" s="3">
-        <v>0.29918784725393172</v>
-      </c>
-      <c r="J4" s="29">
-        <v>0.25239107872812411</v>
-      </c>
-      <c r="K4" s="22" t="s">
+      <c r="G4" s="37">
+        <v>0.40899999999999997</v>
+      </c>
+      <c r="H4" s="37">
+        <v>0.40899999999999997</v>
+      </c>
+      <c r="I4" s="37">
+        <v>0.32100000000000001</v>
+      </c>
+      <c r="J4" s="39">
+        <v>0.27</v>
+      </c>
+      <c r="K4" s="19" t="s">
         <v>9</v>
       </c>
       <c r="L4" s="10">
@@ -1025,31 +1095,31 @@
       <c r="C5" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="D5" s="28" t="s">
+      <c r="D5" s="23" t="s">
         <v>12</v>
       </c>
       <c r="E5" s="3">
-        <v>0.72666306736921149</v>
+        <v>0.74199999999999999</v>
       </c>
       <c r="F5" s="2" t="s">
         <v>15</v>
       </c>
       <c r="G5" s="3">
-        <v>0.47193141512061798</v>
+        <v>0.48699999999999999</v>
       </c>
       <c r="H5" s="3">
-        <v>0.36877739940137788</v>
+        <v>0.35499999999999998</v>
       </c>
       <c r="I5" s="3">
-        <v>0.47193141512061798</v>
-      </c>
-      <c r="J5" s="29">
-        <v>0.15929118547800411</v>
-      </c>
-      <c r="K5" s="22" t="s">
+        <v>0.48699999999999999</v>
+      </c>
+      <c r="J5" s="24">
+        <v>0.158</v>
+      </c>
+      <c r="K5" s="32" t="s">
         <v>13</v>
       </c>
-      <c r="L5" s="10">
+      <c r="L5" s="33">
         <v>0.57726191012009487</v>
       </c>
       <c r="M5" s="7" t="s">
@@ -1069,37 +1139,37 @@
       <c r="C6" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="D6" s="28" t="s">
+      <c r="D6" s="36" t="s">
         <v>16</v>
       </c>
-      <c r="E6" s="3">
-        <v>0.5923278399789782</v>
-      </c>
-      <c r="F6" s="2" t="s">
+      <c r="E6" s="37">
+        <v>0.60499999999999998</v>
+      </c>
+      <c r="F6" s="38" t="s">
         <v>8</v>
       </c>
-      <c r="G6" s="3">
-        <v>0.53434971535753051</v>
-      </c>
-      <c r="H6" s="3">
-        <v>0.53434971535753051</v>
-      </c>
-      <c r="I6" s="3">
-        <v>0.27751904808588018</v>
-      </c>
-      <c r="J6" s="29">
-        <v>0.18813123655658939</v>
-      </c>
-      <c r="K6" s="22" t="s">
+      <c r="G6" s="37">
+        <v>0.52400000000000002</v>
+      </c>
+      <c r="H6" s="37">
+        <v>0.52400000000000002</v>
+      </c>
+      <c r="I6" s="37">
+        <v>0.29899999999999999</v>
+      </c>
+      <c r="J6" s="39">
+        <v>0.17699999999999999</v>
+      </c>
+      <c r="K6" s="32" t="s">
         <v>16</v>
       </c>
-      <c r="L6" s="10">
+      <c r="L6" s="33">
         <v>0.54153527244196309</v>
       </c>
-      <c r="M6" s="7" t="s">
+      <c r="M6" s="34" t="s">
         <v>16</v>
       </c>
-      <c r="N6" s="8">
+      <c r="N6" s="35">
         <v>0.52246509063124191</v>
       </c>
     </row>
@@ -1113,28 +1183,28 @@
       <c r="C7" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="D7" s="28" t="s">
+      <c r="D7" s="23" t="s">
         <v>19</v>
       </c>
       <c r="E7" s="3">
-        <v>0.56656823576215165</v>
+        <v>0.56499999999999995</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>8</v>
+        <v>39</v>
       </c>
       <c r="G7" s="3">
-        <v>0.41946847352738448</v>
+        <v>0.42599999999999999</v>
       </c>
       <c r="H7" s="3">
-        <v>0.41946847352738448</v>
+        <v>0.40300000000000002</v>
       </c>
       <c r="I7" s="3">
-        <v>0.21488670568714599</v>
-      </c>
-      <c r="J7" s="29">
-        <v>0.3656448207854695</v>
-      </c>
-      <c r="K7" s="22" t="s">
+        <v>0.17100000000000001</v>
+      </c>
+      <c r="J7" s="24">
+        <v>0.42599999999999999</v>
+      </c>
+      <c r="K7" s="19" t="s">
         <v>19</v>
       </c>
       <c r="L7" s="10">
@@ -1157,37 +1227,37 @@
       <c r="C8" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="D8" s="28" t="s">
+      <c r="D8" s="23" t="s">
         <v>21</v>
       </c>
       <c r="E8" s="3">
-        <v>0.50140831292591292</v>
+        <v>0.50800000000000001</v>
       </c>
       <c r="F8" s="2" t="s">
         <v>15</v>
       </c>
       <c r="G8" s="3">
-        <v>0.4034698581529681</v>
+        <v>0.39900000000000002</v>
       </c>
       <c r="H8" s="3">
-        <v>0.38792373041708811</v>
+        <v>0.38</v>
       </c>
       <c r="I8" s="3">
-        <v>0.4034698581529681</v>
-      </c>
-      <c r="J8" s="29">
-        <v>0.20860641142994371</v>
-      </c>
-      <c r="K8" s="22" t="s">
+        <v>0.39900000000000002</v>
+      </c>
+      <c r="J8" s="24">
+        <v>0.221</v>
+      </c>
+      <c r="K8" s="19" t="s">
         <v>21</v>
       </c>
       <c r="L8" s="10">
         <v>0.57036701856795147</v>
       </c>
-      <c r="M8" s="7" t="s">
+      <c r="M8" s="34" t="s">
         <v>22</v>
       </c>
-      <c r="N8" s="8">
+      <c r="N8" s="35">
         <v>0.64140582314118721</v>
       </c>
     </row>
@@ -1201,28 +1271,28 @@
       <c r="C9" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="D9" s="28" t="s">
+      <c r="D9" s="23" t="s">
         <v>25</v>
       </c>
       <c r="E9" s="3">
-        <v>0.50318625241944936</v>
+        <v>0.52</v>
       </c>
       <c r="F9" s="2" t="s">
         <v>8</v>
       </c>
       <c r="G9" s="3">
-        <v>0.50723671552945437</v>
+        <v>0.47899999999999998</v>
       </c>
       <c r="H9" s="3">
-        <v>0.50723671552945437</v>
+        <v>0.47899999999999998</v>
       </c>
       <c r="I9" s="3">
-        <v>0.3090391505592302</v>
-      </c>
-      <c r="J9" s="29">
-        <v>0.18372413391131551</v>
-      </c>
-      <c r="K9" s="22" t="s">
+        <v>0.32400000000000001</v>
+      </c>
+      <c r="J9" s="24">
+        <v>0.19700000000000001</v>
+      </c>
+      <c r="K9" s="19" t="s">
         <v>25</v>
       </c>
       <c r="L9" s="10">
@@ -1245,31 +1315,31 @@
       <c r="C10" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="D10" s="28" t="s">
-        <v>28</v>
+      <c r="D10" s="23" t="s">
+        <v>41</v>
       </c>
       <c r="E10" s="3">
-        <v>0.508718310285459</v>
+        <v>0.502</v>
       </c>
       <c r="F10" s="2" t="s">
         <v>8</v>
       </c>
       <c r="G10" s="3">
-        <v>0.55766158029356616</v>
+        <v>0.54800000000000004</v>
       </c>
       <c r="H10" s="3">
-        <v>0.55766158029356616</v>
+        <v>0.54800000000000004</v>
       </c>
       <c r="I10" s="3">
-        <v>0.25521672562135772</v>
-      </c>
-      <c r="J10" s="29">
-        <v>0.1871216940850762</v>
-      </c>
-      <c r="K10" s="22" t="s">
+        <v>0.23799999999999999</v>
+      </c>
+      <c r="J10" s="24">
+        <v>0.21299999999999999</v>
+      </c>
+      <c r="K10" s="32" t="s">
         <v>27</v>
       </c>
-      <c r="L10" s="10">
+      <c r="L10" s="33">
         <v>0.56495442307833654</v>
       </c>
       <c r="M10" s="7" t="s">
@@ -1280,46 +1350,46 @@
       </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A11" s="15" t="s">
+      <c r="A11" s="12" t="s">
         <v>29</v>
       </c>
-      <c r="B11" s="15" t="s">
+      <c r="B11" s="12" t="s">
         <v>30</v>
       </c>
-      <c r="C11" s="20" t="s">
+      <c r="C11" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="D11" s="30" t="s">
+      <c r="D11" s="25" t="s">
+        <v>40</v>
+      </c>
+      <c r="E11" s="13">
+        <v>0.50600000000000001</v>
+      </c>
+      <c r="F11" s="12" t="s">
+        <v>8</v>
+      </c>
+      <c r="G11" s="13">
+        <v>0.44800000000000001</v>
+      </c>
+      <c r="H11" s="13">
+        <v>0.44800000000000001</v>
+      </c>
+      <c r="I11" s="13">
+        <v>0.214</v>
+      </c>
+      <c r="J11" s="26">
+        <v>0.33800000000000002</v>
+      </c>
+      <c r="K11" s="20" t="s">
         <v>29</v>
       </c>
-      <c r="E11" s="16">
-        <v>0.53117529916980721</v>
-      </c>
-      <c r="F11" s="15" t="s">
-        <v>8</v>
-      </c>
-      <c r="G11" s="16">
-        <v>0.46180222001196458</v>
-      </c>
-      <c r="H11" s="16">
-        <v>0.46180222001196458</v>
-      </c>
-      <c r="I11" s="16">
-        <v>0.2354571399123066</v>
-      </c>
-      <c r="J11" s="31">
-        <v>0.30274064007572871</v>
-      </c>
-      <c r="K11" s="23" t="s">
+      <c r="L11" s="14">
+        <v>0.55532067109467609</v>
+      </c>
+      <c r="M11" s="15" t="s">
         <v>29</v>
       </c>
-      <c r="L11" s="17">
-        <v>0.55532067109467609</v>
-      </c>
-      <c r="M11" s="18" t="s">
-        <v>29</v>
-      </c>
-      <c r="N11" s="19">
+      <c r="N11" s="16">
         <v>0.68077962743839049</v>
       </c>
     </row>

</xml_diff>